<commit_message>
push changes why buy not triggerd
</commit_message>
<xml_diff>
--- a/daily_analysis_combined.xlsx
+++ b/daily_analysis_combined.xlsx
@@ -757,8 +757,10 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>102.49368</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>102.49368 stop_loss</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -780,17 +782,17 @@
       <c r="C25" t="n">
         <v>115.62</v>
       </c>
-      <c r="D25" t="n">
-        <v>150</v>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>buy_triggered</t>
         </is>
       </c>
-      <c r="G25" t="n">
-        <v>102.49368</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>102.49368 stop_loss</t>
+        </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -808,12 +810,8 @@
       <c r="C26" t="n">
         <v>94.38</v>
       </c>
-      <c r="D26" t="n">
-        <v>69.63</v>
-      </c>
-      <c r="E26" t="n">
-        <v>69.63</v>
-      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -832,9 +830,7 @@
       <c r="C27" t="n">
         <v>79.25999999999999</v>
       </c>
-      <c r="D27" t="n">
-        <v>105</v>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>

</xml_diff>

<commit_message>
i thin fib is fanalized confirmation from larry is left
</commit_message>
<xml_diff>
--- a/daily_analysis_combined.xlsx
+++ b/daily_analysis_combined.xlsx
@@ -765,7 +765,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>102.49368 stop_loss_1 | trade_closed</t>
+          <t>102.49368 stop_loss_1</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -808,14 +808,10 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>102.49368 stop_loss_2_1 | trade_closed</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>trade_closed</t>
-        </is>
-      </c>
+          <t>150.0 sell_profit_2_1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>trade_closed</t>
@@ -853,7 +849,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>90.81168 stop_loss_2_2 | trade_closed</t>
+          <t>90.81168 stop_loss_2_2</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -1012,7 +1008,7 @@
         <v>115</v>
       </c>
       <c r="H33" t="n">
-        <v>105</v>
+        <v>150</v>
       </c>
       <c r="I33" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
lets work on sell now
</commit_message>
<xml_diff>
--- a/daily_analysis_combined.xlsx
+++ b/daily_analysis_combined.xlsx
@@ -849,7 +849,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>90.81168 stop_loss_2_2</t>
+          <t>171.24 sell_profit_2_2</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -882,8 +882,16 @@
           <t>buy_triggered</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>128.76 sell_profit_3_1</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -909,8 +917,16 @@
           <t>buy_triggered</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>115.62 sell_profit_3_2</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1014,7 +1030,7 @@
         <v>100</v>
       </c>
       <c r="J33" t="n">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="K33" t="n">
         <v>75</v>

</xml_diff>

<commit_message>
in attempt 1 it is confirmed sell working but no pnls now going to add pnl code
</commit_message>
<xml_diff>
--- a/daily_analysis_combined.xlsx
+++ b/daily_analysis_combined.xlsx
@@ -1154,11 +1154,6 @@
           <t>day7</t>
         </is>
       </c>
-      <c r="U59" s="1" t="inlineStr">
-        <is>
-          <t>pnl_point</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1213,7 +1208,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>332.38079999999997 buy_profit_1 ( error1)</t>
+          <t>329.0192 buyback_profit_1</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -1223,9 +1218,6 @@
       </c>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
-      <c r="U60" t="n">
-        <v>-2.719199999999944</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1281,24 +1273,13 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>330.7 buy_profit_2_1 ( error1)</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>trade_closed</t>
-        </is>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>trade_closed</t>
-        </is>
-      </c>
+          <t>328.5 buyback_profit_2_1 ( error1)</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
-      <c r="U61" t="n">
-        <v>-1.680799999999977</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1352,26 +1333,11 @@
           <t>sell_triggered</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>331.73839999999996 buy_profit_2_2 ( error1)</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>trade_closed</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>trade_closed</t>
-        </is>
-      </c>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
-      <c r="U62" t="n">
-        <v>-2.719199999999944</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1426,7 +1392,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>329.6616 buy_profit_3_1 ( error1)</t>
+          <t>328.5 stop_loss_3_1</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -1446,9 +1412,6 @@
       </c>
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr"/>
-      <c r="U63" t="n">
-        <v>-1.680800000000033</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1503,7 +1466,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>329.0192 buy_profit_3_2 ( error1)</t>
+          <t>329.0192 stop_loss_3_2</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -1523,9 +1486,6 @@
       </c>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
-      <c r="U64" t="n">
-        <v>-1.038400000000024</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1578,7 +1538,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>328.5 buy_profit_4 ( error1)</t>
+          <t>327.9808 stop_loss_4</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -1598,9 +1558,6 @@
       </c>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
-      <c r="U65" t="n">
-        <v>-1.258399999999995</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
@@ -1634,97 +1591,97 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>d1_1</t>
+          <t>u1_1</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>329.6616</v>
       </c>
       <c r="C68" t="n">
-        <v>332.3808</v>
+        <v>329.0192</v>
       </c>
       <c r="D68" t="n">
-        <v>328.3774688</v>
+        <v>330.7</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>d2_2_1</t>
+          <t>u2_2_1</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>329.0192</v>
       </c>
       <c r="C69" t="n">
-        <v>330.7</v>
+        <v>328.5</v>
       </c>
       <c r="D69" t="n">
-        <v>328.3774688</v>
+        <v>329.6616</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>d2_2_2</t>
+          <t>u2_2_2</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>329.0192</v>
       </c>
       <c r="C70" t="n">
-        <v>331.7384</v>
+        <v>327.9808</v>
       </c>
       <c r="D70" t="n">
-        <v>327.8063488</v>
+        <v>330.7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>d3_2_1</t>
+          <t>u3_2_1</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>327.9808</v>
       </c>
       <c r="C71" t="n">
-        <v>329.6616</v>
+        <v>327.2416</v>
       </c>
       <c r="D71" t="n">
-        <v>326.7708</v>
+        <v>328.5</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>d3_2_2</t>
+          <t>u3_2_2</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>327.9808</v>
       </c>
       <c r="C72" t="n">
+        <v>326.3</v>
+      </c>
+      <c r="D72" t="n">
         <v>329.0192</v>
-      </c>
-      <c r="D72" t="n">
-        <v>326.7708</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>d1_4</t>
+          <t>u1_4</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>327.2416</v>
       </c>
       <c r="C73" t="n">
-        <v>328.5</v>
+        <v>326.3</v>
       </c>
       <c r="D73" t="n">
-        <v>326.3</v>
+        <v>327.9808</v>
       </c>
     </row>
     <row r="74">
@@ -8374,11 +8331,6 @@
           <t>day7</t>
         </is>
       </c>
-      <c r="U449" s="1" t="inlineStr">
-        <is>
-          <t>pnl_point</t>
-        </is>
-      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -8431,11 +8383,6 @@
       <c r="R450" t="inlineStr"/>
       <c r="S450" t="inlineStr"/>
       <c r="T450" t="inlineStr"/>
-      <c r="U450" t="inlineStr">
-        <is>
-          <t>trade_not_closed</t>
-        </is>
-      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -8494,11 +8441,6 @@
       </c>
       <c r="S451" t="inlineStr"/>
       <c r="T451" t="inlineStr"/>
-      <c r="U451" t="inlineStr">
-        <is>
-          <t>trade_not_closed</t>
-        </is>
-      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -8557,11 +8499,6 @@
       </c>
       <c r="S452" t="inlineStr"/>
       <c r="T452" t="inlineStr"/>
-      <c r="U452" t="inlineStr">
-        <is>
-          <t>trade_not_closed</t>
-        </is>
-      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -8617,7 +8554,7 @@
       </c>
       <c r="P453" t="inlineStr">
         <is>
-          <t>331.6032 buy_profit_3_1 ( error1)</t>
+          <t>329.5132 buyback_profit_3_1 ( error1)</t>
         </is>
       </c>
       <c r="Q453" t="inlineStr">
@@ -8632,9 +8569,6 @@
       </c>
       <c r="S453" t="inlineStr"/>
       <c r="T453" t="inlineStr"/>
-      <c r="U453" t="n">
-        <v>-1.451600000000042</v>
-      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -8688,14 +8622,10 @@
           <t>sell_triggered</t>
         </is>
       </c>
-      <c r="P454" t="inlineStr">
-        <is>
-          <t>331.0484 buy_profit_3_2 ( error1)</t>
-        </is>
-      </c>
+      <c r="P454" t="inlineStr"/>
       <c r="Q454" t="inlineStr">
         <is>
-          <t>trade_closed</t>
+          <t>328.7 buyback_profit_3_2</t>
         </is>
       </c>
       <c r="R454" t="inlineStr">
@@ -8705,9 +8635,6 @@
       </c>
       <c r="S454" t="inlineStr"/>
       <c r="T454" t="inlineStr"/>
-      <c r="U454" t="n">
-        <v>-0.8968000000000416</v>
-      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -8760,7 +8687,7 @@
       </c>
       <c r="O455" t="inlineStr">
         <is>
-          <t>330.6 buy_profit_4 ( error1)</t>
+          <t>330.1516 stop_loss_4</t>
         </is>
       </c>
       <c r="P455" t="inlineStr">
@@ -8780,9 +8707,6 @@
       </c>
       <c r="S455" t="inlineStr"/>
       <c r="T455" t="inlineStr"/>
-      <c r="U455" t="n">
-        <v>-1.086800000000039</v>
-      </c>
     </row>
     <row r="456">
       <c r="A456" s="1" t="inlineStr">
@@ -8816,97 +8740,97 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>d1_1</t>
+          <t>u1_1</t>
         </is>
       </c>
       <c r="B458" t="n">
         <v>331.6032</v>
       </c>
       <c r="C458" t="n">
-        <v>333.9516</v>
+        <v>331.0484</v>
       </c>
       <c r="D458" t="n">
-        <v>330.4941776</v>
+        <v>332.5</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>d2_2_1</t>
+          <t>u2_2_1</t>
         </is>
       </c>
       <c r="B459" t="n">
         <v>331.0484</v>
       </c>
       <c r="C459" t="n">
-        <v>332.5</v>
+        <v>330.6</v>
       </c>
       <c r="D459" t="n">
-        <v>330.4941776</v>
+        <v>331.6032</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>d2_2_2</t>
+          <t>u2_2_2</t>
         </is>
       </c>
       <c r="B460" t="n">
         <v>331.0484</v>
       </c>
       <c r="C460" t="n">
-        <v>333.3968</v>
+        <v>330.1516</v>
       </c>
       <c r="D460" t="n">
-        <v>330.0009376</v>
+        <v>332.5</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>d3_2_1</t>
+          <t>u3_2_1</t>
         </is>
       </c>
       <c r="B461" t="n">
         <v>330.1516</v>
       </c>
       <c r="C461" t="n">
-        <v>331.6032</v>
+        <v>329.5132</v>
       </c>
       <c r="D461" t="n">
-        <v>329.1066</v>
+        <v>330.6</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>d3_2_2</t>
+          <t>u3_2_2</t>
         </is>
       </c>
       <c r="B462" t="n">
         <v>330.1516</v>
       </c>
       <c r="C462" t="n">
+        <v>328.7</v>
+      </c>
+      <c r="D462" t="n">
         <v>331.0484</v>
-      </c>
-      <c r="D462" t="n">
-        <v>329.1066</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>d1_4</t>
+          <t>u1_4</t>
         </is>
       </c>
       <c r="B463" t="n">
         <v>329.5132</v>
       </c>
       <c r="C463" t="n">
-        <v>330.6</v>
+        <v>328.7</v>
       </c>
       <c r="D463" t="n">
-        <v>328.7</v>
+        <v>330.1516</v>
       </c>
     </row>
     <row r="464">

</xml_diff>

<commit_message>
sell is also working and giving pnls just like buy is giving correctly apparently all looking good
</commit_message>
<xml_diff>
--- a/daily_analysis_combined.xlsx
+++ b/daily_analysis_combined.xlsx
@@ -1154,6 +1154,11 @@
           <t>day7</t>
         </is>
       </c>
+      <c r="U59" s="1" t="inlineStr">
+        <is>
+          <t>pnl_point</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1218,6 +1223,9 @@
       </c>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
+      <c r="U60" t="n">
+        <v>0.6424000000000092</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1280,6 +1288,9 @@
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
+      <c r="U61" t="n">
+        <v>0.5192000000000121</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1338,6 +1349,11 @@
       <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>trade_not_closed</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1412,6 +1428,9 @@
       </c>
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr"/>
+      <c r="U63" t="n">
+        <v>-0.5192000000000121</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1486,6 +1505,9 @@
       </c>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
+      <c r="U64" t="n">
+        <v>-1.038400000000024</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1558,6 +1580,9 @@
       </c>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
+      <c r="U65" t="n">
+        <v>-0.7391999999999825</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
@@ -8331,6 +8356,11 @@
           <t>day7</t>
         </is>
       </c>
+      <c r="U449" s="1" t="inlineStr">
+        <is>
+          <t>pnl_point</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -8383,6 +8413,11 @@
       <c r="R450" t="inlineStr"/>
       <c r="S450" t="inlineStr"/>
       <c r="T450" t="inlineStr"/>
+      <c r="U450" t="inlineStr">
+        <is>
+          <t>trade_not_closed</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -8441,6 +8476,11 @@
       </c>
       <c r="S451" t="inlineStr"/>
       <c r="T451" t="inlineStr"/>
+      <c r="U451" t="inlineStr">
+        <is>
+          <t>trade_not_closed</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -8499,6 +8539,11 @@
       </c>
       <c r="S452" t="inlineStr"/>
       <c r="T452" t="inlineStr"/>
+      <c r="U452" t="inlineStr">
+        <is>
+          <t>trade_not_closed</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -8569,6 +8614,9 @@
       </c>
       <c r="S453" t="inlineStr"/>
       <c r="T453" t="inlineStr"/>
+      <c r="U453" t="n">
+        <v>0.6383999999999901</v>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -8635,6 +8683,9 @@
       </c>
       <c r="S454" t="inlineStr"/>
       <c r="T454" t="inlineStr"/>
+      <c r="U454" t="n">
+        <v>1.451599999999985</v>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -8707,6 +8758,9 @@
       </c>
       <c r="S455" t="inlineStr"/>
       <c r="T455" t="inlineStr"/>
+      <c r="U455" t="n">
+        <v>-0.6383999999999901</v>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="1" t="inlineStr">

</xml_diff>

<commit_message>
buy and sell are starting triggereing and giving TP/SL from current day ( working )
</commit_message>
<xml_diff>
--- a/daily_analysis_combined.xlsx
+++ b/daily_analysis_combined.xlsx
@@ -1208,12 +1208,12 @@
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>sell_triggered</t>
+          <t>sell_triggered_329.0192_buyback_profit_1</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>329.0192 buyback_profit_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -1224,7 +1224,7 @@
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
       <c r="U60" t="n">
-        <v>0.6424000000000092</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="61">
@@ -1276,20 +1276,16 @@
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr">
         <is>
-          <t>sell_triggered</t>
-        </is>
-      </c>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>328.5 buyback_profit_2_1 ( error1)</t>
-        </is>
-      </c>
+          <t>sell_triggered_328.5_buyback_profit_2_1</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
       <c r="U61" t="n">
-        <v>0.5192000000000121</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="62">
@@ -1403,12 +1399,12 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>sell_triggered</t>
+          <t>sell_triggered_327.2416_buyback_profit_3_1</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>328.5 stop_loss_3_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -1429,7 +1425,7 @@
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="n">
-        <v>-0.5192000000000121</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="64">
@@ -1506,7 +1502,7 @@
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="n">
-        <v>-1.038400000000024</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="65">
@@ -1555,12 +1551,12 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>sell_triggered</t>
+          <t>sell_triggered_327.9808_stop_loss_4</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>327.9808 stop_loss_4</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -1581,7 +1577,7 @@
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="n">
-        <v>-0.7391999999999825</v>
+        <v>-0.74</v>
       </c>
     </row>
     <row r="66">
@@ -2398,21 +2394,33 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O125" t="inlineStr"/>
-      <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr"/>
+          <t>buy_triggered_328.552532_stop_loss_1</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>331.73699999999997 sell_profit_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr"/>
       <c r="U125" t="n">
-        <v>2.16</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="126">
@@ -2463,12 +2471,12 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_328.552532_stop_loss_2_1</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>330.4 sell_profit_2_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -2489,7 +2497,7 @@
       <c r="S126" t="inlineStr"/>
       <c r="T126" t="inlineStr"/>
       <c r="U126" t="n">
-        <v>1.34</v>
+        <v>-0.51</v>
       </c>
     </row>
     <row r="127">
@@ -2694,12 +2702,12 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_329.063_sell_profit_3_2</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>329.063 sell_profit_3_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
@@ -4778,12 +4786,12 @@
       </c>
       <c r="N255" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_330.624684_stop_loss_1</t>
         </is>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>330.624684 stop_loss_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
@@ -4855,12 +4863,12 @@
       </c>
       <c r="N256" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_330.624684_stop_loss_2_1</t>
         </is>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>330.624684 stop_loss_2_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
@@ -4932,12 +4940,12 @@
       </c>
       <c r="N257" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_330.040584_stop_loss_2_2</t>
         </is>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>330.040584 stop_loss_2_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
@@ -5009,13 +5017,17 @@
       </c>
       <c r="N258" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O258" t="inlineStr"/>
+          <t>buy_triggered_328.9815_stop_loss_3_1</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>331.938 sell_profit_3_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
@@ -5031,7 +5043,7 @@
       <c r="S258" t="inlineStr"/>
       <c r="T258" t="inlineStr"/>
       <c r="U258" t="n">
-        <v>1.72</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="259">
@@ -5082,13 +5094,17 @@
       </c>
       <c r="N259" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O259" t="inlineStr"/>
+          <t>buy_triggered_328.9815_stop_loss_3_2</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>331.281 sell_profit_3_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -5104,7 +5120,7 @@
       <c r="S259" t="inlineStr"/>
       <c r="T259" t="inlineStr"/>
       <c r="U259" t="n">
-        <v>1.06</v>
+        <v>-1.24</v>
       </c>
     </row>
     <row r="260">
@@ -5153,13 +5169,17 @@
       </c>
       <c r="N260" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O260" t="inlineStr"/>
+          <t>buy_triggered_328.5_stop_loss_4</t>
+        </is>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>330.75 sell_profit_4</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -5175,7 +5195,7 @@
       <c r="S260" t="inlineStr"/>
       <c r="T260" t="inlineStr"/>
       <c r="U260" t="n">
-        <v>1.29</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="261">
@@ -5992,12 +6012,12 @@
       </c>
       <c r="N320" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_331.27455760000004_stop_loss_1</t>
         </is>
       </c>
       <c r="O320" t="inlineStr">
         <is>
-          <t>331.27455760000004 stop_loss_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P320" t="inlineStr">
@@ -6069,15 +6089,19 @@
       </c>
       <c r="N321" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_331.27455760000004_stop_loss_2_1</t>
         </is>
       </c>
       <c r="O321" t="inlineStr">
         <is>
-          <t>331.27455760000004 stop_loss_2_1</t>
-        </is>
-      </c>
-      <c r="P321" t="inlineStr"/>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="Q321" t="inlineStr">
         <is>
           <t>trade_closed</t>
@@ -6142,14 +6166,22 @@
       </c>
       <c r="N322" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O322" t="inlineStr"/>
-      <c r="P322" t="inlineStr"/>
+          <t>buy_triggered_330.4568176_stop_loss_2_2</t>
+        </is>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="Q322" t="inlineStr">
         <is>
-          <t>330.4568176 stop_loss_2_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="R322" t="inlineStr">
@@ -6211,12 +6243,12 @@
       </c>
       <c r="N323" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_328.9741_stop_loss_3_1</t>
         </is>
       </c>
       <c r="O323" t="inlineStr">
         <is>
-          <t>333.1132 sell_profit_3_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P323" t="inlineStr">
@@ -6237,7 +6269,7 @@
       <c r="S323" t="inlineStr"/>
       <c r="T323" t="inlineStr"/>
       <c r="U323" t="n">
-        <v>2.41</v>
+        <v>-1.73</v>
       </c>
     </row>
     <row r="324">
@@ -6288,12 +6320,12 @@
       </c>
       <c r="N324" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_328.9741_stop_loss_3_2</t>
         </is>
       </c>
       <c r="O324" t="inlineStr">
         <is>
-          <t>332.1934 sell_profit_3_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P324" t="inlineStr">
@@ -6314,7 +6346,7 @@
       <c r="S324" t="inlineStr"/>
       <c r="T324" t="inlineStr"/>
       <c r="U324" t="n">
-        <v>1.49</v>
+        <v>-1.73</v>
       </c>
     </row>
     <row r="325">
@@ -6363,12 +6395,12 @@
       </c>
       <c r="N325" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_331.45000000000005_sell_profit_4</t>
         </is>
       </c>
       <c r="O325" t="inlineStr">
         <is>
-          <t>331.45000000000005 sell_profit_4</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P325" t="inlineStr">
@@ -7206,12 +7238,12 @@
       </c>
       <c r="N385" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_331.4440512_stop_loss_1</t>
         </is>
       </c>
       <c r="O385" t="inlineStr">
         <is>
-          <t>331.4440512 stop_loss_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P385" t="inlineStr">
@@ -7283,12 +7315,12 @@
       </c>
       <c r="N386" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_331.4440512_stop_loss_2_1</t>
         </is>
       </c>
       <c r="O386" t="inlineStr">
         <is>
-          <t>331.4440512 stop_loss_2_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P386" t="inlineStr">
@@ -7360,12 +7392,12 @@
       </c>
       <c r="N387" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_330.7171712_stop_loss_2_2</t>
         </is>
       </c>
       <c r="O387" t="inlineStr">
         <is>
-          <t>330.7171712 stop_loss_2_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P387" t="inlineStr">
@@ -7437,15 +7469,27 @@
       </c>
       <c r="N388" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O388" t="inlineStr"/>
-      <c r="P388" t="inlineStr"/>
-      <c r="Q388" t="inlineStr"/>
+          <t>buy_triggered_329.3992_stop_loss_3_1</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="P388" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="Q388" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="R388" t="inlineStr">
         <is>
-          <t>329.3992 stop_loss_3_1</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="S388" t="inlineStr"/>
@@ -7502,15 +7546,27 @@
       </c>
       <c r="N389" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
-        </is>
-      </c>
-      <c r="O389" t="inlineStr"/>
-      <c r="P389" t="inlineStr"/>
-      <c r="Q389" t="inlineStr"/>
+          <t>buy_triggered_329.3992_stop_loss_3_2</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="P389" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
+      <c r="Q389" t="inlineStr">
+        <is>
+          <t>trade_closed</t>
+        </is>
+      </c>
       <c r="R389" t="inlineStr">
         <is>
-          <t>329.3992 stop_loss_3_2</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="S389" t="inlineStr"/>
@@ -7565,12 +7621,12 @@
       </c>
       <c r="N390" t="inlineStr">
         <is>
-          <t>buy_triggered</t>
+          <t>buy_triggered_331.6_sell_profit_4</t>
         </is>
       </c>
       <c r="O390" t="inlineStr">
         <is>
-          <t>331.6 sell_profit_4</t>
+          <t>trade_closed</t>
         </is>
       </c>
       <c r="P390" t="inlineStr">
@@ -8471,15 +8527,13 @@
       <c r="Q451" t="inlineStr"/>
       <c r="R451" t="inlineStr">
         <is>
-          <t>sell_triggered</t>
+          <t>sell_triggered_330.6_buyback_profit_2_1</t>
         </is>
       </c>
       <c r="S451" t="inlineStr"/>
       <c r="T451" t="inlineStr"/>
-      <c r="U451" t="inlineStr">
-        <is>
-          <t>trade_not_closed</t>
-        </is>
+      <c r="U451" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="452">
@@ -8594,14 +8648,10 @@
       <c r="N453" t="inlineStr"/>
       <c r="O453" t="inlineStr">
         <is>
-          <t>sell_triggered</t>
-        </is>
-      </c>
-      <c r="P453" t="inlineStr">
-        <is>
-          <t>329.5132 buyback_profit_3_1 ( error1)</t>
-        </is>
-      </c>
+          <t>sell_triggered_329.5132_buyback_profit_3_1</t>
+        </is>
+      </c>
+      <c r="P453" t="inlineStr"/>
       <c r="Q453" t="inlineStr">
         <is>
           <t>trade_closed</t>
@@ -8615,7 +8665,7 @@
       <c r="S453" t="inlineStr"/>
       <c r="T453" t="inlineStr"/>
       <c r="U453" t="n">
-        <v>0.6383999999999901</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="454">
@@ -8684,7 +8734,7 @@
       <c r="S454" t="inlineStr"/>
       <c r="T454" t="inlineStr"/>
       <c r="U454" t="n">
-        <v>1.451599999999985</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="455">
@@ -8759,7 +8809,7 @@
       <c r="S455" t="inlineStr"/>
       <c r="T455" t="inlineStr"/>
       <c r="U455" t="n">
-        <v>-0.6383999999999901</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="456">

</xml_diff>